<commit_message>
PAUSED (task177): stage 4 fixes, waiting on round 2 readers
Round 1 (target.zip 2c536aaa): judge DETERMINISTIC / APPROVE; both scored readers missed the call (11, 13) and
kept 5 and 14 of 24 ask figures. Own-use primary re-sited onto the vendor's support desk in the staff console
(accounts registered to the supplier's GST/HST number on the invoices), the employer widget's UTC now moves every
month (employers' month-end filings), and plan 1.3 files release 4.0's resolution for the app, the web and the
voice service. The call (26), the stump and every call-side figure are unchanged; checks 109 of 109, verify 25 of
25, byte-identical rebuild, figures_check and precut exit 0.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01A6XcFx5t62c7gPi1bBKcVi
</commit_message>
<xml_diff>
--- a/task177/golden/assistant_share_forecast_mar_apr_2027.xlsx
+++ b/task177/golden/assistant_share_forecast_mar_apr_2027.xlsx
@@ -226,7 +226,7 @@
     <t>2026</t>
   </si>
   <si>
-    <t>A conversation counts once, in the month its first session started, Manitoba time. The test employers registered to our own business number are our own use; the employer widget writes UTC, moved here to Manitoba time.</t>
+    <t>A conversation counts once, in the month its first session started, Manitoba time. The test employers registered to our own business number are our own use; the employer widget writes UTC, moved here to Manitoba time. Riverlot's support desk works in the staff console under accounts registered to Riverlot's business number; those conversations are the vendor's and are not counted.</t>
   </si>
   <si>
     <t>As of</t>
@@ -1260,7 +1260,7 @@
         <v>42</v>
       </c>
       <c r="B2" s="3">
-        <v>930</v>
+        <v>945</v>
       </c>
       <c r="C2" s="3">
         <v>1256</v>
@@ -1271,7 +1271,7 @@
         <v>43</v>
       </c>
       <c r="B3" s="3">
-        <v>1020</v>
+        <v>1040</v>
       </c>
       <c r="C3" s="3">
         <v>1148</v>
@@ -1282,7 +1282,7 @@
         <v>44</v>
       </c>
       <c r="B4" s="3">
-        <v>1519</v>
+        <v>1555</v>
       </c>
       <c r="C4" s="3">
         <v>1326</v>
@@ -1293,7 +1293,7 @@
         <v>45</v>
       </c>
       <c r="B5" s="3">
-        <v>1656</v>
+        <v>1686</v>
       </c>
       <c r="C5" s="3">
         <v>1171</v>
@@ -1304,7 +1304,7 @@
         <v>46</v>
       </c>
       <c r="B6" s="3">
-        <v>1840</v>
+        <v>1850</v>
       </c>
       <c r="C6" s="3">
         <v>1163</v>
@@ -1315,7 +1315,7 @@
         <v>47</v>
       </c>
       <c r="B7" s="3">
-        <v>1815</v>
+        <v>1852</v>
       </c>
       <c r="C7" s="3">
         <v>1217</v>
@@ -1326,7 +1326,7 @@
         <v>48</v>
       </c>
       <c r="B8" s="3">
-        <v>1621</v>
+        <v>1660</v>
       </c>
       <c r="C8" s="3">
         <v>1332</v>
@@ -1337,7 +1337,7 @@
         <v>49</v>
       </c>
       <c r="B9" s="3">
-        <v>1360</v>
+        <v>1399</v>
       </c>
       <c r="C9" s="3">
         <v>1161</v>
@@ -1348,7 +1348,7 @@
         <v>50</v>
       </c>
       <c r="B10" s="3">
-        <v>1811</v>
+        <v>1838</v>
       </c>
       <c r="C10" s="3">
         <v>1224</v>
@@ -1359,7 +1359,7 @@
         <v>51</v>
       </c>
       <c r="B11" s="3">
-        <v>1772</v>
+        <v>1794</v>
       </c>
       <c r="C11" s="3">
         <v>1208</v>
@@ -1370,7 +1370,7 @@
         <v>52</v>
       </c>
       <c r="B12" s="3">
-        <v>1760</v>
+        <v>1799</v>
       </c>
       <c r="C12" s="3">
         <v>1252</v>
@@ -1381,7 +1381,7 @@
         <v>53</v>
       </c>
       <c r="B13" s="3">
-        <v>1172</v>
+        <v>1203</v>
       </c>
       <c r="C13" s="3">
         <v>1244</v>
@@ -1392,7 +1392,7 @@
         <v>66</v>
       </c>
       <c r="B14" s="10">
-        <v>18276</v>
+        <v>18621</v>
       </c>
       <c r="C14" s="10">
         <v>14702</v>

</xml_diff>

<commit_message>
PAUSED (task177): stage 4 round 3 fix, waiting on the re-judge
Round 3 (target.zip 8ab100af): readers E and F missed the call (13, 11) and kept 0 of 24 ask figures; the judge
NOT_DETERMINISTIC on the whole per cent (its reproductions ran 25.8 to 27.9 under open conventions). The share is
now asked to the nearest 5 per cent (golden 26.05 prints 25, 1.45 points inside its cell); plan 5.1 files the
denominator and the start channel, plan 4.1 the check-in's due date; the learner, its rates and the transfers'
weighting stay unfiled. Every judge reading under the filed conventions prints 25 or is ruled out (J3 in checks).
Moved: the call 26 to 25 (and two workbook-only model forecasts). Checks 130 of 130, verify 26 of 26,
byte-identical rebuild, figures_check and precut exit 0; heart BLOCK ruled by the author (window fixed at draw).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01A6XcFx5t62c7gPi1bBKcVi
</commit_message>
<xml_diff>
--- a/task177/golden/assistant_share_forecast_mar_apr_2027.xlsx
+++ b/task177/golden/assistant_share_forecast_mar_apr_2027.xlsx
@@ -31,7 +31,7 @@
     <t>Digital Channels, prepared 5 January 2027 for the March and April usage tier</t>
   </si>
   <si>
-    <t>Forecast share started in Ask Prairie Works (whole per cent)</t>
+    <t>Forecast share started in Ask Prairie Works (nearest 5 per cent)</t>
   </si>
   <si>
     <t>Jobseekers on the register on 3 January 2027</t>
@@ -79,7 +79,7 @@
     <t>Learning rate, overflow transfers</t>
   </si>
   <si>
-    <t>One learning rate for every contact would give (whole per cent)</t>
+    <t>One learning rate for every contact would give (nearest 5 per cent)</t>
   </si>
   <si>
     <t>Model</t>
@@ -106,7 +106,7 @@
     <t>Pull to last choice</t>
   </si>
   <si>
-    <t>Forecast share (whole per cent)</t>
+    <t>Forecast share (nearest 5 per cent)</t>
   </si>
   <si>
     <t>Separate rate for overflow transfers (used)</t>
@@ -265,7 +265,7 @@
     <t>Rounding</t>
   </si>
   <si>
-    <t>Shares to the whole per cent, rounded once from the unrounded forecast; counts whole.</t>
+    <t>The forecast shares to the nearest 5 per cent, rounded once from the unrounded forecast; the 2026 record's shares to the whole per cent; counts whole.</t>
   </si>
   <si>
     <t>Sources</t>
@@ -674,7 +674,7 @@
         <v>2</v>
       </c>
       <c r="B4" s="1">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
@@ -851,7 +851,7 @@
         <v>0.31</v>
       </c>
       <c r="I2" s="8">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
@@ -938,7 +938,7 @@
         <v>0</v>
       </c>
       <c r="I5" s="8">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
@@ -967,7 +967,7 @@
         <v>0.28</v>
       </c>
       <c r="I6" s="8">
-        <v>28</v>
+        <v>30</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">

</xml_diff>